<commit_message>
fix: script & margin
</commit_message>
<xml_diff>
--- a/data_set/expense.xlsx
+++ b/data_set/expense.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FMIS\Tech-project\R20-dashboard\data_set\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E09524-B217-4C94-B4C6-D94020E78DAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9C3E0F-70E0-4B25-8A85-DDE7F57501D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
   <si>
     <t xml:space="preserve">   </t>
   </si>
@@ -131,9 +131,6 @@
   </si>
   <si>
     <t>Q4</t>
-  </si>
-  <si>
-    <t>(-10393900000000)</t>
   </si>
   <si>
     <t>EXPENDITURE_CATEGORY</t>
@@ -633,14 +630,14 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="5">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="5">
-        <v>217578000000</v>
+        <v>217577900000</v>
       </c>
       <c r="D2" s="5">
         <v>1240000000</v>
@@ -649,68 +646,68 @@
         <v>0</v>
       </c>
       <c r="F2" s="5">
-        <v>218818000000</v>
+        <v>218817900000</v>
       </c>
       <c r="G2" s="5">
-        <v>42864977654</v>
+        <v>48209095942</v>
       </c>
       <c r="H2" s="5">
         <f>F2-G2</f>
-        <v>175953022346</v>
+        <v>170608804058</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="5">
-        <v>21388100000000</v>
+        <v>21402185349565</v>
       </c>
       <c r="D3" s="5">
-        <v>726039000000</v>
+        <v>727558067731</v>
       </c>
       <c r="E3" s="5">
-        <v>7173000000000</v>
+        <v>7172995437000</v>
       </c>
       <c r="F3" s="5">
-        <v>29287200000000</v>
+        <v>29302738854296</v>
       </c>
       <c r="G3" s="5">
-        <v>28376355807847</v>
+        <v>29179286624080</v>
       </c>
       <c r="H3" s="5">
         <f t="shared" ref="H3" si="0">F3-G3</f>
-        <v>910844192153</v>
+        <v>123452230216</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>4</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="5">
-        <v>17654600000000</v>
+        <v>6709555205670</v>
       </c>
       <c r="D4" s="5">
-        <v>1016670000000</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>30</v>
+        <v>876380975700</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0</v>
       </c>
       <c r="F4" s="5">
-        <v>8277340000000</v>
+        <v>7585936181370</v>
       </c>
       <c r="G4" s="5">
-        <v>7277340000000</v>
+        <v>6945568413215</v>
       </c>
       <c r="H4" s="5">
         <f>F4-G4</f>
-        <v>1000000000000</v>
+        <v>640367768155</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -722,27 +719,27 @@
       </c>
       <c r="C5" s="5">
         <f>SUM(C2:C4)</f>
-        <v>39260278000000</v>
+        <v>28329318455235</v>
       </c>
       <c r="D5" s="5">
         <f t="shared" ref="D5:H5" si="1">SUM(D2:D4)</f>
-        <v>1743949000000</v>
+        <v>1605179043431</v>
       </c>
       <c r="E5" s="5">
         <f>SUM(E2:E4)</f>
-        <v>7173000000000</v>
+        <v>7172995437000</v>
       </c>
       <c r="F5" s="5">
         <f>SUM(F2:F4)</f>
-        <v>37783358000000</v>
+        <v>37107492935666</v>
       </c>
       <c r="G5" s="5">
         <f t="shared" si="1"/>
-        <v>35696560785501</v>
+        <v>36173064133237</v>
       </c>
       <c r="H5" s="5">
         <f t="shared" si="1"/>
-        <v>2086797214499</v>
+        <v>934428802429</v>
       </c>
     </row>
   </sheetData>
@@ -916,7 +913,7 @@
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.5" customWidth="1"/>
     <col min="3" max="3" width="30.375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -925,7 +922,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>9</v>
@@ -936,7 +933,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="5">
         <v>4146836925880</v>
@@ -947,7 +944,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="5">
         <v>10291599273634</v>
@@ -958,7 +955,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="5">
         <v>5911962313874</v>
@@ -969,7 +966,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="5">
         <v>5446626292405</v>
@@ -997,13 +994,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1011,7 +1008,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C2" s="5">
         <v>1999012198073</v>
@@ -1025,7 +1022,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" s="5">
         <v>3798910478175</v>
@@ -1039,7 +1036,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="5">
         <v>748213160596</v>
@@ -1053,7 +1050,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="5">
         <v>551623172986</v>
@@ -1067,7 +1064,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="5">
         <v>11633686827512</v>
@@ -1081,7 +1078,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" s="5">
         <v>4451772018</v>

</xml_diff>

<commit_message>
feat: update data and graphs
</commit_message>
<xml_diff>
--- a/data_set/expense.xlsx
+++ b/data_set/expense.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FMIS\Tech-project\R20-dashboard\data_set\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104002E7-A80E-47B5-941F-9A749589DECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F150BC-BC17-4452-BEC9-DE8806D3A591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="Sheet 3 " sheetId="4" r:id="rId3"/>
     <sheet name="Sheet 4" sheetId="5" r:id="rId4"/>
     <sheet name="Sheet 5" sheetId="6" r:id="rId5"/>
+    <sheet name="M_2025" sheetId="7" r:id="rId6"/>
+    <sheet name="Q_2025" sheetId="9" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$H$5</definedName>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="42">
   <si>
     <t xml:space="preserve">   </t>
   </si>
@@ -131,6 +133,42 @@
   </si>
   <si>
     <t>Social Sector</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Dec</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
   </si>
 </sst>
 </file>
@@ -198,7 +236,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -208,7 +246,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -595,19 +640,19 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="5">
         <v>19124997642364</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="5">
         <v>76190226</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="5">
         <v>4786188100000</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="5">
         <v>23911261932590</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="5">
         <v>7138347419054</v>
       </c>
       <c r="H2" s="5">
@@ -622,19 +667,19 @@
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="5">
         <v>6546712545966.2998</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="5">
         <v>510735414838</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="5">
         <v>0</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="5">
         <v>7057447960804.2998</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="5">
         <v>888965801579</v>
       </c>
       <c r="H3" s="5">
@@ -650,27 +695,27 @@
         <v>14</v>
       </c>
       <c r="C4" s="5">
-        <f>SUM(C2:C3)</f>
+        <f t="shared" ref="C4:H4" si="0">SUM(C2:C3)</f>
         <v>25671710188330.301</v>
       </c>
       <c r="D4" s="5">
-        <f>SUM(D2:D3)</f>
+        <f t="shared" si="0"/>
         <v>510811605064</v>
       </c>
       <c r="E4" s="5">
-        <f>SUM(E2:E3)</f>
+        <f t="shared" si="0"/>
         <v>4786188100000</v>
       </c>
       <c r="F4" s="5">
-        <f>SUM(F2:F3)</f>
+        <f t="shared" si="0"/>
         <v>30968709893394.301</v>
       </c>
       <c r="G4" s="5">
-        <f>SUM(G2:G3)</f>
+        <f t="shared" si="0"/>
         <v>8027313220633</v>
       </c>
       <c r="H4" s="5">
-        <f>SUM(H2:H3)</f>
+        <f t="shared" si="0"/>
         <v>22941396672761.301</v>
       </c>
     </row>
@@ -708,7 +753,7 @@
       <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="5">
         <v>5138276519193</v>
       </c>
     </row>
@@ -719,7 +764,7 @@
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="5">
         <v>1843527924376</v>
       </c>
     </row>
@@ -730,7 +775,7 @@
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="5">
         <v>1045508777064</v>
       </c>
     </row>
@@ -768,7 +813,7 @@
       <c r="B2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="5">
         <v>438644389901</v>
       </c>
     </row>
@@ -779,7 +824,7 @@
       <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="5">
         <v>4233714551255</v>
       </c>
     </row>
@@ -790,7 +835,7 @@
       <c r="B4" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="5">
         <v>1087646623554</v>
       </c>
     </row>
@@ -801,7 +846,7 @@
       <c r="B5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="5">
         <v>850940739922</v>
       </c>
     </row>
@@ -842,10 +887,10 @@
       <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="5">
         <v>2283155862062</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="5">
         <v>11679312508124</v>
       </c>
     </row>
@@ -856,10 +901,10 @@
       <c r="B3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="5">
         <v>379419917269</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="5">
         <v>5672564188205.2998</v>
       </c>
     </row>
@@ -870,10 +915,10 @@
       <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="5">
         <v>561086105282</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="5">
         <v>2031613285768</v>
       </c>
     </row>
@@ -884,10 +929,10 @@
       <c r="B5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="5">
         <v>154089364654</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="5">
         <v>770830000000</v>
       </c>
     </row>
@@ -898,10 +943,10 @@
       <c r="B6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="5">
         <v>4589530471366</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="5">
         <v>10659320225983</v>
       </c>
     </row>
@@ -912,10 +957,10 @@
       <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="5">
         <v>0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="5">
         <v>148370835000</v>
       </c>
     </row>
@@ -952,7 +997,7 @@
       <c r="B2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="5">
         <v>7967281720633</v>
       </c>
     </row>
@@ -960,4 +1005,232 @@
   <autoFilter ref="A1:C2" xr:uid="{3C422C38-199D-42CF-BC1B-FCE487D9B7BD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B790029-151D-439F-826B-A8E5EC5D528B}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.375" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="19.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="10">
+        <v>5082745134684</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="10">
+        <v>2020939931173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="10">
+        <v>3501085853043</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="10">
+        <v>1950327370548</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="10">
+        <v>2113506905289</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="10">
+        <v>3087685652641</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="10">
+        <v>2630278673333</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="10">
+        <v>2807689736601</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="9">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="10">
+        <v>3052095146708</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="9">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="10">
+        <v>2521353748586</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="9">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="10">
+        <v>2349698835425</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="9">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="10">
+        <v>5007448049264</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A5EA846-6351-46DD-B0EF-044698DA304B}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="13">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="14">
+        <v>10536172381870</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="13">
+        <v>2</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="14">
+        <v>6987599928478</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
+        <v>3</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="14">
+        <v>8411062756642</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="13">
+        <v>4</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="14">
+        <v>9374547833275</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>